<commit_message>
fix: update variant handling and template size retention in import history fix: improve template size assignment logic in price tag processing fix: adjust strike line color in A5 price tag template chore: update POP price tag template file
</commit_message>
<xml_diff>
--- a/public/templates/pricetag/Template POP Price Tag.xlsx
+++ b/public/templates/pricetag/Template POP Price Tag.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\price-tag\public\templates\pricetag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF3C0008-1F58-481E-905B-B364AAE49402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DA21319-B9F4-4E71-A9EC-60FE4552668E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{54CCA4BC-3671-4B73-81DD-38D59B3891BB}"/>
+    <workbookView xWindow="4890" yWindow="3570" windowWidth="21600" windowHeight="11295" xr2:uid="{54CCA4BC-3671-4B73-81DD-38D59B3891BB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -112,11 +112,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -457,7 +461,7 @@
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
-    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" style="3" customWidth="1"/>
     <col min="4" max="4" width="34.5703125" customWidth="1"/>
     <col min="5" max="5" width="24.140625" customWidth="1"/>
     <col min="6" max="6" width="40.42578125" customWidth="1"/>
@@ -471,7 +475,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">

</xml_diff>

<commit_message>
Improve table header layout and update product name in manual entry
</commit_message>
<xml_diff>
--- a/public/templates/pricetag/Template POP Price Tag.xlsx
+++ b/public/templates/pricetag/Template POP Price Tag.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\price-tag\public\templates\pricetag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF3C0008-1F58-481E-905B-B364AAE49402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C592DC-2A80-4F05-98B5-BF0A9B2B9573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{54CCA4BC-3671-4B73-81DD-38D59B3891BB}"/>
   </bookViews>
@@ -50,20 +50,20 @@
     <t>SKU/PLU</t>
   </si>
   <si>
-    <t>Brand/Merk</t>
-  </si>
-  <si>
     <t>Harga Normal (Rp)</t>
   </si>
   <si>
-    <t>Diskon (%) / Harga Promo (Rp)</t>
+    <t>Nama Produk</t>
+  </si>
+  <si>
+    <t>Program Promo (Rp / %)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -85,6 +85,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Constantia"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -99,7 +104,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -107,16 +112,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -452,19 +469,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F62F10-8D49-4EA4-A515-A56735334A18}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22.7109375" customWidth="1"/>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
     <col min="3" max="3" width="21.28515625" customWidth="1"/>
-    <col min="4" max="4" width="34.5703125" customWidth="1"/>
-    <col min="5" max="5" width="24.140625" customWidth="1"/>
+    <col min="4" max="4" width="74" customWidth="1"/>
+    <col min="5" max="5" width="25.42578125" customWidth="1"/>
     <col min="6" max="6" width="40.42578125" customWidth="1"/>
     <col min="7" max="7" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,14 +492,17 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+    </row>
+    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D2" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: update Template POP Price Tag.xlsx with new content
</commit_message>
<xml_diff>
--- a/public/templates/pricetag/Template POP Price Tag.xlsx
+++ b/public/templates/pricetag/Template POP Price Tag.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\price-tag\public\templates\pricetag\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C592DC-2A80-4F05-98B5-BF0A9B2B9573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{717538B6-6DA4-43D9-BEA2-58F7F1B5F780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{54CCA4BC-3671-4B73-81DD-38D59B3891BB}"/>
   </bookViews>
@@ -104,23 +104,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color auto="1"/>
-      </top>
-      <bottom style="medium">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -133,7 +122,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Bad" xfId="1" builtinId="27"/>
@@ -481,7 +470,7 @@
     <col min="7" max="7" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -501,7 +490,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="D2" s="2"/>
     </row>
   </sheetData>

</xml_diff>